<commit_message>
docs: fase 2 inconsistencias resueltas en su mayoria y fase 3 generado un modelo de dominio consolidado
- fase 2 inconsistencias resueltas en su mayoria
- fase 3 generado un modelo de dominio consolidado (falta cuzarlo con las inconsistencias de la fase2)
</commit_message>
<xml_diff>
--- a/fases-y-plan-de-trabajo/fase2/Revisar inconsitencias .xlsx
+++ b/fases-y-plan-de-trabajo/fase2/Revisar inconsitencias .xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gogyt\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lfgon\OneDrive\Documentos\GitHub\proyecto-llm\fases-y-plan-de-trabajo\fase2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46620B1-61DC-4F39-9107-4FDA1A5606A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5E78EE-4A52-4173-801E-A2383ED1F4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B60F64C-3736-4759-8FFE-77C70AD4AEAE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{1B60F64C-3736-4759-8FFE-77C70AD4AEAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Inconsistencias" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="95">
   <si>
     <t>Column1</t>
   </si>
@@ -101,9 +101,6 @@
     <t>contradicción entre fuentes</t>
   </si>
   <si>
-    <t>null</t>
-  </si>
-  <si>
     <t>HC-002</t>
   </si>
   <si>
@@ -252,13 +249,100 @@
   </si>
   <si>
     <t>Sección 2.14: "Los tramos definidos son hasta dos mil validaciones mensuales, de dos mil a cinco mil, y sobre cinco mil." | ENT4 Francisca Leiva [00:03:07]: "Si una validación es un documento, son cuarenta mil. Si es un caso, son doce mil. En ningún escenario son dos mil." | ENT8 Valentina Ruiz-Tagle [00:15:16]: "Los tramos están definidos hasta diez mil validaciones mensuales y hay un tramo que dice "diez mil o más" sin precio. Ese es el tramo en el que va a caer el cliente piloto."</t>
+  </si>
+  <si>
+    <t>Se fija el umbral de aprobación automática en 90 puntos, alineado con lo solicitado por el cliente piloto. Se corrige la inconsistencia interna del documento (85 vs 80). El umbral queda configurable por cliente y se recalibrará con datos de la marcha blanca.</t>
+  </si>
+  <si>
+    <t>Definido: umbral = 90 puntos</t>
+  </si>
+  <si>
+    <t>Se adopta el plazo de retención de la aseguradora (5 años, hasta 10 según producto) por sobre el default de 90 días. Evidencia en almacenamiento activo los primeros 90 días y luego archivo frío hasta cumplir el plazo correspondiente.</t>
+  </si>
+  <si>
+    <t>Definido: retención 5-10 años según producto</t>
+  </si>
+  <si>
+    <t>Se define un modo de carga por lote (bulk) con límite propio para cargas masivas predecibles (histórico inicial, catch-up tras caídas). Para tráfico estándar, exceso de límite = rechazo con cabecera Retry-After.</t>
+  </si>
+  <si>
+    <t>Definido</t>
+  </si>
+  <si>
+    <t>Se mantiene el criterio de la propuesta comercial ya enviada al cliente: se cobra únicamente cuando la plataforma resuelve el caso de forma automática. Casos derivados a revisión humana no se facturan.</t>
+  </si>
+  <si>
+    <t>Definido: se respeta lo comprometido por escrito</t>
+  </si>
+  <si>
+    <t>Pendiente de definir en conjunto con el área de riesgo del cliente piloto. Se agenda reunión de trabajo dedicada antes de cerrar la especificación.</t>
+  </si>
+  <si>
+    <t>Pendiente – requiere reunión con cliente</t>
+  </si>
+  <si>
+    <t>La autenticación contra el directorio corporativo del cliente (SSO) se trata como requisito duro del proyecto, no opcional. Se incorpora formalmente al alcance y cronograma.</t>
+  </si>
+  <si>
+    <t>Definido: SSO obligatorio</t>
+  </si>
+  <si>
+    <t>La escritura de resultados en el sistema de siniestros del cliente se automatiza (no transcripción manual), vía el mismo mecanismo de intercambio de archivos definido en HC-013.</t>
+  </si>
+  <si>
+    <t>Definido: escritura automática vía archivos</t>
+  </si>
+  <si>
+    <t>Se elimina la opción de rechazo automático para el tramo bajo 60 puntos. Todo caso en ese tramo se escala obligatoriamente a un analista humano, quien debe justificar la decisión.</t>
+  </si>
+  <si>
+    <t>Definido, según lo solicitado por Daniela</t>
+  </si>
+  <si>
+    <t>Se cobra una validación por caso, salvo que exista evidencia nueva sustantiva que gatille un reanálisis completo, en cuyo caso se cobra una segunda validación. Regla a documentar formalmente antes de la marcha blanca.</t>
+  </si>
+  <si>
+    <t>Se identifica que el compromiso comercial de "operar en enero" requiere aclaración: definir si implica lanzamiento productivo completo o un piloto supervisado de volumen acotado, reconciliando con el cronograma formal (producción en abril).</t>
+  </si>
+  <si>
+    <t>Pendiente – requiere aclaración con Rodrigo/cliente</t>
+  </si>
+  <si>
+    <t>El SLA se redefine por tramos según tipo/tamaño de archivo en lugar de un número único de 5 segundos. Se deja constancia de que los valores exactos por tramo aún no pueden comprometerse por falta de pruebas de carga suficientes.</t>
+  </si>
+  <si>
+    <t>Definido en estructura; valores exactos pendientes de pruebas</t>
+  </si>
+  <si>
+    <t>Se separa el rastro de decisión (metadato: quién, cuándo, score, decisión), que se mantiene inalterable, del contenido personal de la evidencia, que puede anonimizarse ante una solicitud válida del titular sin eliminar el registro de que la decisión existió.</t>
+  </si>
+  <si>
+    <t>Definido, según propuesta de Daniela</t>
+  </si>
+  <si>
+    <t>La plataforma soporta ambos patrones de integración: API REST para clientes que la expongan, e intercambio de archivos para clientes cuyo core no expone servicios web (caso del cliente piloto).</t>
+  </si>
+  <si>
+    <t>Definido: ambos modos soportados</t>
+  </si>
+  <si>
+    <t>Se redefine "reconstruir una decisión pasada" como trazabilidad completa (inputs, versión de modelo, parámetros y lógica vigentes en ese momento), no como reproducibilidad exacta del output de modelos generativos no deterministas.</t>
+  </si>
+  <si>
+    <t>La meta de 2 semanas para producción aplica a clientes sin formulario personalizado. Para clientes con formulario propio, se comunica un plazo adicional realista de 2-3 semanas para esa configuración.</t>
+  </si>
+  <si>
+    <t>Se propone mantener los tramos actuales y agregar un único tramo nuevo con precio fijo (5.000-15.000), suficiente para cubrir al cliente piloto bajo cualquiera de las dos definiciones de "validación". Sobre 15.000 queda como tramo Enterprise/a convenir en vez de precio fijo, hasta contar con más datos de costo real.</t>
+  </si>
+  <si>
+    <t>Pendiente de validar con finanzas/comercial; depende de resolver definición de "validación" (documento vs caso)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +354,12 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -295,13 +385,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -371,7 +460,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -687,15 +776,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEBD8109-7ECD-4AE1-AA02-E1E1F3282DDC}">
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="176.140625" customWidth="1"/>
-    <col min="3" max="3" width="251" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="3" max="3" width="30.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="6" max="6" width="28.42578125" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -715,347 +806,348 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="375" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="330" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="315" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="225" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="300" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="330" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="B9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="270" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="375" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="390" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="360" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="405" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="345" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="F15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="390" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="F16" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="330" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="F17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>16</v>
+      <c r="D18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1066,7 +1158,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91319C62-10A4-467A-A2F4-805A680E7550}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>